<commit_message>
v1.4: Store Floor v3 — the store in 3D with the team at work
- 3D store from the printed plan (modules/store-floor/planogram.yaml), weekly numbers on every shelf
- shelly/storefloor.py: SKU placement, per-fixture KPIs and status, python -m shelly store
- v3 day simulation: trading hours, two 8h shifts, staggered breaks, Tue/Thu/Sat deliveries,
  Duty Manager directing the team, till cover, jobs from Shelly data, customers peaking after 5pm
- back of house: storeroom, walk-in chiller, office, staff room, restrooms, dock; A* pathfinding
- HQ-style Tasks / Team / Day panels; launchpad card and Floor link in the nav; 12 new tests

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FY9TJhN1QamgkQ7ezStAcj
</commit_message>
<xml_diff>
--- a/docs/reports/Shelly_13_Week_Forecast.xlsx
+++ b/docs/reports/Shelly_13_Week_Forecast.xlsx
@@ -10151,17 +10151,17 @@
     <x v="104"/>
     <x v="3"/>
     <x v="1"/>
-    <n v="3021.21"/>
-    <n v="2758.04"/>
-    <n v="3284.39"/>
+    <n v="3011.37"/>
+    <n v="2749.05"/>
+    <n v="3273.69"/>
   </r>
   <r>
     <x v="104"/>
     <x v="4"/>
     <x v="1"/>
-    <n v="3349.66"/>
-    <n v="3057.87"/>
-    <n v="3641.44"/>
+    <n v="3346.78"/>
+    <n v="3055.25"/>
+    <n v="3638.32"/>
   </r>
   <r>
     <x v="104"/>
@@ -10175,41 +10175,41 @@
     <x v="104"/>
     <x v="6"/>
     <x v="1"/>
-    <n v="1974.96"/>
+    <n v="1974.95"/>
     <n v="1802.92"/>
-    <n v="2147"/>
+    <n v="2146.99"/>
   </r>
   <r>
     <x v="104"/>
     <x v="7"/>
     <x v="1"/>
-    <n v="350.18"/>
-    <n v="319.68"/>
-    <n v="380.68"/>
+    <n v="348.38"/>
+    <n v="318.03"/>
+    <n v="378.72"/>
   </r>
   <r>
     <x v="104"/>
     <x v="8"/>
     <x v="1"/>
-    <n v="549.05"/>
-    <n v="501.23"/>
-    <n v="596.88"/>
+    <n v="550.13"/>
+    <n v="502.21"/>
+    <n v="598.05"/>
   </r>
   <r>
     <x v="104"/>
     <x v="9"/>
     <x v="1"/>
-    <n v="387.48"/>
-    <n v="353.73"/>
-    <n v="421.24"/>
+    <n v="428.58"/>
+    <n v="391.24"/>
+    <n v="465.91"/>
   </r>
   <r>
     <x v="104"/>
     <x v="10"/>
     <x v="1"/>
-    <n v="2025.64"/>
-    <n v="1849.18"/>
-    <n v="2202.09"/>
+    <n v="2024.42"/>
+    <n v="1848.08"/>
+    <n v="2200.77"/>
   </r>
   <r>
     <x v="105"/>
@@ -10239,17 +10239,17 @@
     <x v="105"/>
     <x v="3"/>
     <x v="1"/>
-    <n v="3142.92"/>
-    <n v="2869.14"/>
-    <n v="3416.7"/>
+    <n v="3137.8"/>
+    <n v="2864.47"/>
+    <n v="3411.13"/>
   </r>
   <r>
     <x v="105"/>
     <x v="4"/>
     <x v="1"/>
-    <n v="3472.82"/>
-    <n v="3170.3"/>
-    <n v="3775.33"/>
+    <n v="3471.33"/>
+    <n v="3168.94"/>
+    <n v="3773.72"/>
   </r>
   <r>
     <x v="105"/>
@@ -10265,39 +10265,39 @@
     <x v="1"/>
     <n v="1727.29"/>
     <n v="1576.83"/>
-    <n v="1877.76"/>
+    <n v="1877.75"/>
   </r>
   <r>
     <x v="105"/>
     <x v="7"/>
     <x v="1"/>
-    <n v="380.76"/>
-    <n v="347.59"/>
-    <n v="413.92"/>
+    <n v="379.78"/>
+    <n v="346.69"/>
+    <n v="412.86"/>
   </r>
   <r>
     <x v="105"/>
     <x v="8"/>
     <x v="1"/>
-    <n v="523.51"/>
-    <n v="477.91"/>
-    <n v="569.11"/>
+    <n v="524.02"/>
+    <n v="478.37"/>
+    <n v="569.67"/>
   </r>
   <r>
     <x v="105"/>
     <x v="9"/>
     <x v="1"/>
-    <n v="521.5"/>
-    <n v="476.07"/>
-    <n v="566.9299999999999"/>
+    <n v="548.46"/>
+    <n v="500.68"/>
+    <n v="596.23"/>
   </r>
   <r>
     <x v="105"/>
     <x v="10"/>
     <x v="1"/>
-    <n v="2109.95"/>
-    <n v="1926.15"/>
-    <n v="2293.75"/>
+    <n v="2109.32"/>
+    <n v="1925.58"/>
+    <n v="2293.06"/>
   </r>
   <r>
     <x v="106"/>
@@ -10327,17 +10327,17 @@
     <x v="106"/>
     <x v="3"/>
     <x v="1"/>
-    <n v="3221.88"/>
-    <n v="2941.22"/>
-    <n v="3502.53"/>
+    <n v="3219.25"/>
+    <n v="2938.82"/>
+    <n v="3499.68"/>
   </r>
   <r>
     <x v="106"/>
     <x v="4"/>
     <x v="1"/>
-    <n v="3557.03"/>
-    <n v="3247.18"/>
-    <n v="3866.88"/>
+    <n v="3556.27"/>
+    <n v="3246.48"/>
+    <n v="3866.05"/>
   </r>
   <r>
     <x v="106"/>
@@ -10352,40 +10352,40 @@
     <x v="6"/>
     <x v="1"/>
     <n v="2026.47"/>
-    <n v="1849.95"/>
-    <n v="2203"/>
+    <n v="1849.94"/>
+    <n v="2202.99"/>
   </r>
   <r>
     <x v="106"/>
     <x v="7"/>
     <x v="1"/>
-    <n v="393.62"/>
-    <n v="359.33"/>
-    <n v="427.91"/>
+    <n v="393.11"/>
+    <n v="358.87"/>
+    <n v="427.36"/>
   </r>
   <r>
     <x v="106"/>
     <x v="8"/>
     <x v="1"/>
-    <n v="638.34"/>
-    <n v="582.73"/>
-    <n v="693.9400000000001"/>
+    <n v="638.65"/>
+    <n v="583.02"/>
+    <n v="694.28"/>
   </r>
   <r>
     <x v="106"/>
     <x v="9"/>
     <x v="1"/>
-    <n v="437.41"/>
-    <n v="399.3"/>
-    <n v="475.51"/>
+    <n v="448.57"/>
+    <n v="409.49"/>
+    <n v="487.64"/>
   </r>
   <r>
     <x v="106"/>
     <x v="10"/>
     <x v="1"/>
-    <n v="2011.55"/>
-    <n v="1836.33"/>
-    <n v="2186.78"/>
+    <n v="2011.25"/>
+    <n v="1836.05"/>
+    <n v="2186.45"/>
   </r>
   <r>
     <x v="107"/>
@@ -20452,17 +20452,17 @@
     <x v="104"/>
     <x v="3"/>
     <x v="1"/>
-    <n v="3021.21"/>
-    <n v="2758.04"/>
-    <n v="3284.39"/>
+    <n v="3011.37"/>
+    <n v="2749.05"/>
+    <n v="3273.69"/>
   </r>
   <r>
     <x v="104"/>
     <x v="4"/>
     <x v="1"/>
-    <n v="3349.66"/>
-    <n v="3057.87"/>
-    <n v="3641.44"/>
+    <n v="3346.78"/>
+    <n v="3055.25"/>
+    <n v="3638.32"/>
   </r>
   <r>
     <x v="104"/>
@@ -20476,41 +20476,41 @@
     <x v="104"/>
     <x v="6"/>
     <x v="1"/>
-    <n v="1974.96"/>
+    <n v="1974.95"/>
     <n v="1802.92"/>
-    <n v="2147"/>
+    <n v="2146.99"/>
   </r>
   <r>
     <x v="104"/>
     <x v="7"/>
     <x v="1"/>
-    <n v="350.18"/>
-    <n v="319.68"/>
-    <n v="380.68"/>
+    <n v="348.38"/>
+    <n v="318.03"/>
+    <n v="378.72"/>
   </r>
   <r>
     <x v="104"/>
     <x v="8"/>
     <x v="1"/>
-    <n v="549.05"/>
-    <n v="501.23"/>
-    <n v="596.88"/>
+    <n v="550.13"/>
+    <n v="502.21"/>
+    <n v="598.05"/>
   </r>
   <r>
     <x v="104"/>
     <x v="9"/>
     <x v="1"/>
-    <n v="387.48"/>
-    <n v="353.73"/>
-    <n v="421.24"/>
+    <n v="428.58"/>
+    <n v="391.24"/>
+    <n v="465.91"/>
   </r>
   <r>
     <x v="104"/>
     <x v="10"/>
     <x v="1"/>
-    <n v="2025.64"/>
-    <n v="1849.18"/>
-    <n v="2202.09"/>
+    <n v="2024.42"/>
+    <n v="1848.08"/>
+    <n v="2200.77"/>
   </r>
   <r>
     <x v="105"/>
@@ -20540,17 +20540,17 @@
     <x v="105"/>
     <x v="3"/>
     <x v="1"/>
-    <n v="3142.92"/>
-    <n v="2869.14"/>
-    <n v="3416.7"/>
+    <n v="3137.8"/>
+    <n v="2864.47"/>
+    <n v="3411.13"/>
   </r>
   <r>
     <x v="105"/>
     <x v="4"/>
     <x v="1"/>
-    <n v="3472.82"/>
-    <n v="3170.3"/>
-    <n v="3775.33"/>
+    <n v="3471.33"/>
+    <n v="3168.94"/>
+    <n v="3773.72"/>
   </r>
   <r>
     <x v="105"/>
@@ -20566,39 +20566,39 @@
     <x v="1"/>
     <n v="1727.29"/>
     <n v="1576.83"/>
-    <n v="1877.76"/>
+    <n v="1877.75"/>
   </r>
   <r>
     <x v="105"/>
     <x v="7"/>
     <x v="1"/>
-    <n v="380.76"/>
-    <n v="347.59"/>
-    <n v="413.92"/>
+    <n v="379.78"/>
+    <n v="346.69"/>
+    <n v="412.86"/>
   </r>
   <r>
     <x v="105"/>
     <x v="8"/>
     <x v="1"/>
-    <n v="523.51"/>
-    <n v="477.91"/>
-    <n v="569.11"/>
+    <n v="524.02"/>
+    <n v="478.37"/>
+    <n v="569.67"/>
   </r>
   <r>
     <x v="105"/>
     <x v="9"/>
     <x v="1"/>
-    <n v="521.5"/>
-    <n v="476.07"/>
-    <n v="566.9299999999999"/>
+    <n v="548.46"/>
+    <n v="500.68"/>
+    <n v="596.23"/>
   </r>
   <r>
     <x v="105"/>
     <x v="10"/>
     <x v="1"/>
-    <n v="2109.95"/>
-    <n v="1926.15"/>
-    <n v="2293.75"/>
+    <n v="2109.32"/>
+    <n v="1925.58"/>
+    <n v="2293.06"/>
   </r>
   <r>
     <x v="106"/>
@@ -20628,17 +20628,17 @@
     <x v="106"/>
     <x v="3"/>
     <x v="1"/>
-    <n v="3221.88"/>
-    <n v="2941.22"/>
-    <n v="3502.53"/>
+    <n v="3219.25"/>
+    <n v="2938.82"/>
+    <n v="3499.68"/>
   </r>
   <r>
     <x v="106"/>
     <x v="4"/>
     <x v="1"/>
-    <n v="3557.03"/>
-    <n v="3247.18"/>
-    <n v="3866.88"/>
+    <n v="3556.27"/>
+    <n v="3246.48"/>
+    <n v="3866.05"/>
   </r>
   <r>
     <x v="106"/>
@@ -20653,40 +20653,40 @@
     <x v="6"/>
     <x v="1"/>
     <n v="2026.47"/>
-    <n v="1849.95"/>
-    <n v="2203"/>
+    <n v="1849.94"/>
+    <n v="2202.99"/>
   </r>
   <r>
     <x v="106"/>
     <x v="7"/>
     <x v="1"/>
-    <n v="393.62"/>
-    <n v="359.33"/>
-    <n v="427.91"/>
+    <n v="393.11"/>
+    <n v="358.87"/>
+    <n v="427.36"/>
   </r>
   <r>
     <x v="106"/>
     <x v="8"/>
     <x v="1"/>
-    <n v="638.34"/>
-    <n v="582.73"/>
-    <n v="693.9400000000001"/>
+    <n v="638.65"/>
+    <n v="583.02"/>
+    <n v="694.28"/>
   </r>
   <r>
     <x v="106"/>
     <x v="9"/>
     <x v="1"/>
-    <n v="437.41"/>
-    <n v="399.3"/>
-    <n v="475.51"/>
+    <n v="448.57"/>
+    <n v="409.49"/>
+    <n v="487.64"/>
   </r>
   <r>
     <x v="106"/>
     <x v="10"/>
     <x v="1"/>
-    <n v="2011.55"/>
-    <n v="1836.33"/>
-    <n v="2186.78"/>
+    <n v="2011.25"/>
+    <n v="1836.05"/>
+    <n v="2186.45"/>
   </r>
   <r>
     <x v="107"/>
@@ -22609,22 +22609,22 @@
     <row r="10">
       <c r="B10" s="10">
         <f>Model!$C$21</f>
-        <v>275759.19</v>
+        <v>275812.14</v>
       </c>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="10">
         <f>Model!$D$21</f>
-        <v>251737.96</v>
+        <v>251786.29</v>
       </c>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="10">
         <f>Model!$E$21</f>
-        <v>299780.44</v>
+        <v>299837.99</v>
       </c>
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="11">
         <f>Model!$G$21</f>
-        <v>0.0355811574148071</v>
+        <v>0.0357800049030272</v>
       </c>
       <c r="M10" s="9" t="n"/>
     </row>
@@ -22667,12 +22667,12 @@
     <row r="14">
       <c r="B14" s="10">
         <f>Model!$C$8</f>
-        <v>19074.99</v>
+        <v>19101.42</v>
       </c>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="10">
         <f>Model!$I$21</f>
-        <v>275759.19</v>
+        <v>275812.14</v>
       </c>
       <c r="G14" s="9" t="n"/>
       <c r="H14" s="10">
@@ -22877,15 +22877,15 @@
       </c>
       <c r="C8" s="15">
         <f>SUMIFS(Raw!$D$2:$D$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B8)</f>
-        <v>19074.99</v>
+        <v>19101.42</v>
       </c>
       <c r="D8" s="15">
         <f>SUMIFS(Raw!$E$2:$E$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B8)</f>
-        <v>17413.39</v>
+        <v>17437.52</v>
       </c>
       <c r="E8" s="15">
         <f>SUMIFS(Raw!$F$2:$F$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B8)</f>
-        <v>20736.61</v>
+        <v>20765.34</v>
       </c>
       <c r="F8" s="15">
         <f>SUMIFS(Raw!$D$2:$D$1288,Raw!$C$2:$C$1288,"Actual",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B8-364)</f>
@@ -22893,7 +22893,7 @@
       </c>
       <c r="G8" s="16">
         <f>IFERROR(C8/F8-1,0)</f>
-        <v>-0.0125099396168279</v>
+        <v>-0.0111416892378799</v>
       </c>
       <c r="H8" s="15">
         <f>C8*Assumptions!$C$6</f>
@@ -22901,7 +22901,7 @@
       </c>
       <c r="I8" s="15">
         <f>C8+H8</f>
-        <v>19074.99</v>
+        <v>19101.42</v>
       </c>
     </row>
     <row r="9">
@@ -22910,15 +22910,15 @@
       </c>
       <c r="C9" s="15">
         <f>SUMIFS(Raw!$D$2:$D$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B9)</f>
-        <v>19744.73</v>
+        <v>19763.98</v>
       </c>
       <c r="D9" s="15">
         <f>SUMIFS(Raw!$E$2:$E$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B9)</f>
-        <v>18024.77</v>
+        <v>18042.34</v>
       </c>
       <c r="E9" s="15">
         <f>SUMIFS(Raw!$F$2:$F$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B9)</f>
-        <v>21464.7</v>
+        <v>21485.62</v>
       </c>
       <c r="F9" s="15">
         <f>SUMIFS(Raw!$D$2:$D$1288,Raw!$C$2:$C$1288,"Actual",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B9-364)</f>
@@ -22926,7 +22926,7 @@
       </c>
       <c r="G9" s="16">
         <f>IFERROR(C9/F9-1,0)</f>
-        <v>0.0140546975589939</v>
+        <v>0.0150433437915842</v>
       </c>
       <c r="H9" s="15">
         <f>C9*Assumptions!$C$6</f>
@@ -22934,7 +22934,7 @@
       </c>
       <c r="I9" s="15">
         <f>C9+H9</f>
-        <v>19744.73</v>
+        <v>19763.98</v>
       </c>
     </row>
     <row r="10">
@@ -22943,15 +22943,15 @@
       </c>
       <c r="C10" s="15">
         <f>SUMIFS(Raw!$D$2:$D$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B10)</f>
-        <v>19580.28</v>
+        <v>19587.55</v>
       </c>
       <c r="D10" s="15">
         <f>SUMIFS(Raw!$E$2:$E$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B10)</f>
-        <v>17874.64</v>
+        <v>17881.27</v>
       </c>
       <c r="E10" s="15">
         <f>SUMIFS(Raw!$F$2:$F$1288,Raw!$C$2:$C$1288,"Forecast",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B10)</f>
-        <v>21285.9</v>
+        <v>21293.8</v>
       </c>
       <c r="F10" s="15">
         <f>SUMIFS(Raw!$D$2:$D$1288,Raw!$C$2:$C$1288,"Actual",Raw!$B$2:$B$1288,CatCrit,Raw!$A$2:$A$1288,$B10-364)</f>
@@ -22959,7 +22959,7 @@
       </c>
       <c r="G10" s="16">
         <f>IFERROR(C10/F10-1,0)</f>
-        <v>0.0290884130926765</v>
+        <v>0.0294705053182822</v>
       </c>
       <c r="H10" s="15">
         <f>C10*Assumptions!$C$6</f>
@@ -22967,7 +22967,7 @@
       </c>
       <c r="I10" s="15">
         <f>C10+H10</f>
-        <v>19580.28</v>
+        <v>19587.55</v>
       </c>
     </row>
     <row r="11">
@@ -23308,15 +23308,15 @@
       </c>
       <c r="C21" s="18">
         <f>SUM(C8:C20)</f>
-        <v>275759.19</v>
+        <v>275812.14</v>
       </c>
       <c r="D21" s="18">
         <f>SUM(D8:D20)</f>
-        <v>251737.96</v>
+        <v>251786.29</v>
       </c>
       <c r="E21" s="18">
         <f>SUM(E8:E20)</f>
-        <v>299780.44</v>
+        <v>299837.99</v>
       </c>
       <c r="F21" s="18">
         <f>SUM(F8:F20)</f>
@@ -23324,7 +23324,7 @@
       </c>
       <c r="G21" s="19">
         <f>IFERROR(C21/F21-1,0)</f>
-        <v>0.0355811574148071</v>
+        <v>0.0357800049030272</v>
       </c>
       <c r="H21" s="18">
         <f>SUM(H8:H20)</f>
@@ -23332,7 +23332,7 @@
       </c>
       <c r="I21" s="18">
         <f>SUM(I8:I20)</f>
-        <v>275759.19</v>
+        <v>275812.14</v>
       </c>
     </row>
     <row r="24">
@@ -23774,7 +23774,7 @@
         </is>
       </c>
       <c r="B12" s="20" t="n">
-        <v>370031.67</v>
+        <v>370014.08</v>
       </c>
     </row>
     <row r="13">
@@ -23784,7 +23784,7 @@
         </is>
       </c>
       <c r="B13" s="20" t="n">
-        <v>408834.13</v>
+        <v>408829</v>
       </c>
     </row>
     <row r="14">
@@ -23804,7 +23804,7 @@
         </is>
       </c>
       <c r="B15" s="20" t="n">
-        <v>221406.88</v>
+        <v>221406.87</v>
       </c>
     </row>
     <row r="16">
@@ -23814,7 +23814,7 @@
         </is>
       </c>
       <c r="B16" s="20" t="n">
-        <v>38321.37</v>
+        <v>38318.08</v>
       </c>
     </row>
     <row r="17">
@@ -23824,7 +23824,7 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>61743.21</v>
+        <v>61745.11</v>
       </c>
     </row>
     <row r="18">
@@ -23834,7 +23834,7 @@
         </is>
       </c>
       <c r="B18" s="20" t="n">
-        <v>52598.12</v>
+        <v>52677.34</v>
       </c>
     </row>
     <row r="19">
@@ -23844,7 +23844,7 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>228181.31</v>
+        <v>228179.16</v>
       </c>
     </row>
     <row r="20">
@@ -23854,7 +23854,7 @@
         </is>
       </c>
       <c r="B20" s="20" t="n">
-        <v>2281599.02</v>
+        <v>2281651.97</v>
       </c>
     </row>
     <row r="24">
@@ -25572,10 +25572,10 @@
         <v>0</v>
       </c>
       <c r="C131" s="20" t="n">
-        <v>19074.99</v>
+        <v>19101.42</v>
       </c>
       <c r="D131" s="20" t="n">
-        <v>19074.99</v>
+        <v>19101.42</v>
       </c>
     </row>
     <row r="132">
@@ -25588,10 +25588,10 @@
         <v>0</v>
       </c>
       <c r="C132" s="20" t="n">
-        <v>19744.73</v>
+        <v>19763.98</v>
       </c>
       <c r="D132" s="20" t="n">
-        <v>19744.73</v>
+        <v>19763.98</v>
       </c>
     </row>
     <row r="133">
@@ -25604,10 +25604,10 @@
         <v>0</v>
       </c>
       <c r="C133" s="20" t="n">
-        <v>19580.28</v>
+        <v>19587.55</v>
       </c>
       <c r="D133" s="20" t="n">
-        <v>19580.28</v>
+        <v>19587.55</v>
       </c>
     </row>
     <row r="134">
@@ -25780,10 +25780,10 @@
         <v>2005839.83</v>
       </c>
       <c r="C144" s="20" t="n">
-        <v>275759.1900000001</v>
+        <v>275812.14</v>
       </c>
       <c r="D144" s="20" t="n">
-        <v>2281599.02</v>
+        <v>2281651.97</v>
       </c>
     </row>
   </sheetData>
@@ -48808,13 +48808,13 @@
         </is>
       </c>
       <c r="D1149" s="24" t="n">
-        <v>3021.21</v>
+        <v>3011.37</v>
       </c>
       <c r="E1149" s="24" t="n">
-        <v>2758.04</v>
+        <v>2749.05</v>
       </c>
       <c r="F1149" s="24" t="n">
-        <v>3284.39</v>
+        <v>3273.69</v>
       </c>
     </row>
     <row r="1150">
@@ -48832,13 +48832,13 @@
         </is>
       </c>
       <c r="D1150" s="24" t="n">
-        <v>3349.66</v>
+        <v>3346.78</v>
       </c>
       <c r="E1150" s="24" t="n">
-        <v>3057.87</v>
+        <v>3055.25</v>
       </c>
       <c r="F1150" s="24" t="n">
-        <v>3641.44</v>
+        <v>3638.32</v>
       </c>
     </row>
     <row r="1151">
@@ -48880,13 +48880,13 @@
         </is>
       </c>
       <c r="D1152" s="24" t="n">
-        <v>1974.96</v>
+        <v>1974.95</v>
       </c>
       <c r="E1152" s="24" t="n">
         <v>1802.92</v>
       </c>
       <c r="F1152" s="24" t="n">
-        <v>2147</v>
+        <v>2146.99</v>
       </c>
     </row>
     <row r="1153">
@@ -48904,13 +48904,13 @@
         </is>
       </c>
       <c r="D1153" s="24" t="n">
-        <v>350.18</v>
+        <v>348.38</v>
       </c>
       <c r="E1153" s="24" t="n">
-        <v>319.68</v>
+        <v>318.03</v>
       </c>
       <c r="F1153" s="24" t="n">
-        <v>380.68</v>
+        <v>378.72</v>
       </c>
     </row>
     <row r="1154">
@@ -48928,13 +48928,13 @@
         </is>
       </c>
       <c r="D1154" s="24" t="n">
-        <v>549.05</v>
+        <v>550.13</v>
       </c>
       <c r="E1154" s="24" t="n">
-        <v>501.23</v>
+        <v>502.21</v>
       </c>
       <c r="F1154" s="24" t="n">
-        <v>596.88</v>
+        <v>598.05</v>
       </c>
     </row>
     <row r="1155">
@@ -48952,13 +48952,13 @@
         </is>
       </c>
       <c r="D1155" s="24" t="n">
-        <v>387.48</v>
+        <v>428.58</v>
       </c>
       <c r="E1155" s="24" t="n">
-        <v>353.73</v>
+        <v>391.24</v>
       </c>
       <c r="F1155" s="24" t="n">
-        <v>421.24</v>
+        <v>465.91</v>
       </c>
     </row>
     <row r="1156">
@@ -48976,13 +48976,13 @@
         </is>
       </c>
       <c r="D1156" s="24" t="n">
-        <v>2025.64</v>
+        <v>2024.42</v>
       </c>
       <c r="E1156" s="24" t="n">
-        <v>1849.18</v>
+        <v>1848.08</v>
       </c>
       <c r="F1156" s="24" t="n">
-        <v>2202.09</v>
+        <v>2200.77</v>
       </c>
     </row>
     <row r="1157">
@@ -49072,13 +49072,13 @@
         </is>
       </c>
       <c r="D1160" s="24" t="n">
-        <v>3142.92</v>
+        <v>3137.8</v>
       </c>
       <c r="E1160" s="24" t="n">
-        <v>2869.14</v>
+        <v>2864.47</v>
       </c>
       <c r="F1160" s="24" t="n">
-        <v>3416.7</v>
+        <v>3411.13</v>
       </c>
     </row>
     <row r="1161">
@@ -49096,13 +49096,13 @@
         </is>
       </c>
       <c r="D1161" s="24" t="n">
-        <v>3472.82</v>
+        <v>3471.33</v>
       </c>
       <c r="E1161" s="24" t="n">
-        <v>3170.3</v>
+        <v>3168.94</v>
       </c>
       <c r="F1161" s="24" t="n">
-        <v>3775.33</v>
+        <v>3773.72</v>
       </c>
     </row>
     <row r="1162">
@@ -49150,7 +49150,7 @@
         <v>1576.83</v>
       </c>
       <c r="F1163" s="24" t="n">
-        <v>1877.76</v>
+        <v>1877.75</v>
       </c>
     </row>
     <row r="1164">
@@ -49168,13 +49168,13 @@
         </is>
       </c>
       <c r="D1164" s="24" t="n">
-        <v>380.76</v>
+        <v>379.78</v>
       </c>
       <c r="E1164" s="24" t="n">
-        <v>347.59</v>
+        <v>346.69</v>
       </c>
       <c r="F1164" s="24" t="n">
-        <v>413.92</v>
+        <v>412.86</v>
       </c>
     </row>
     <row r="1165">
@@ -49192,13 +49192,13 @@
         </is>
       </c>
       <c r="D1165" s="24" t="n">
-        <v>523.51</v>
+        <v>524.02</v>
       </c>
       <c r="E1165" s="24" t="n">
-        <v>477.91</v>
+        <v>478.37</v>
       </c>
       <c r="F1165" s="24" t="n">
-        <v>569.11</v>
+        <v>569.67</v>
       </c>
     </row>
     <row r="1166">
@@ -49216,13 +49216,13 @@
         </is>
       </c>
       <c r="D1166" s="24" t="n">
-        <v>521.5</v>
+        <v>548.46</v>
       </c>
       <c r="E1166" s="24" t="n">
-        <v>476.07</v>
+        <v>500.68</v>
       </c>
       <c r="F1166" s="24" t="n">
-        <v>566.9299999999999</v>
+        <v>596.23</v>
       </c>
     </row>
     <row r="1167">
@@ -49240,13 +49240,13 @@
         </is>
       </c>
       <c r="D1167" s="24" t="n">
-        <v>2109.95</v>
+        <v>2109.32</v>
       </c>
       <c r="E1167" s="24" t="n">
-        <v>1926.15</v>
+        <v>1925.58</v>
       </c>
       <c r="F1167" s="24" t="n">
-        <v>2293.75</v>
+        <v>2293.06</v>
       </c>
     </row>
     <row r="1168">
@@ -49336,13 +49336,13 @@
         </is>
       </c>
       <c r="D1171" s="24" t="n">
-        <v>3221.88</v>
+        <v>3219.25</v>
       </c>
       <c r="E1171" s="24" t="n">
-        <v>2941.22</v>
+        <v>2938.82</v>
       </c>
       <c r="F1171" s="24" t="n">
-        <v>3502.53</v>
+        <v>3499.68</v>
       </c>
     </row>
     <row r="1172">
@@ -49360,13 +49360,13 @@
         </is>
       </c>
       <c r="D1172" s="24" t="n">
-        <v>3557.03</v>
+        <v>3556.27</v>
       </c>
       <c r="E1172" s="24" t="n">
-        <v>3247.18</v>
+        <v>3246.48</v>
       </c>
       <c r="F1172" s="24" t="n">
-        <v>3866.88</v>
+        <v>3866.05</v>
       </c>
     </row>
     <row r="1173">
@@ -49411,10 +49411,10 @@
         <v>2026.47</v>
       </c>
       <c r="E1174" s="24" t="n">
-        <v>1849.95</v>
+        <v>1849.94</v>
       </c>
       <c r="F1174" s="24" t="n">
-        <v>2203</v>
+        <v>2202.99</v>
       </c>
     </row>
     <row r="1175">
@@ -49432,13 +49432,13 @@
         </is>
       </c>
       <c r="D1175" s="24" t="n">
-        <v>393.62</v>
+        <v>393.11</v>
       </c>
       <c r="E1175" s="24" t="n">
-        <v>359.33</v>
+        <v>358.87</v>
       </c>
       <c r="F1175" s="24" t="n">
-        <v>427.91</v>
+        <v>427.36</v>
       </c>
     </row>
     <row r="1176">
@@ -49456,13 +49456,13 @@
         </is>
       </c>
       <c r="D1176" s="24" t="n">
-        <v>638.34</v>
+        <v>638.65</v>
       </c>
       <c r="E1176" s="24" t="n">
-        <v>582.73</v>
+        <v>583.02</v>
       </c>
       <c r="F1176" s="24" t="n">
-        <v>693.9400000000001</v>
+        <v>694.28</v>
       </c>
     </row>
     <row r="1177">
@@ -49480,13 +49480,13 @@
         </is>
       </c>
       <c r="D1177" s="24" t="n">
-        <v>437.41</v>
+        <v>448.57</v>
       </c>
       <c r="E1177" s="24" t="n">
-        <v>399.3</v>
+        <v>409.49</v>
       </c>
       <c r="F1177" s="24" t="n">
-        <v>475.51</v>
+        <v>487.64</v>
       </c>
     </row>
     <row r="1178">
@@ -49504,13 +49504,13 @@
         </is>
       </c>
       <c r="D1178" s="24" t="n">
-        <v>2011.55</v>
+        <v>2011.25</v>
       </c>
       <c r="E1178" s="24" t="n">
-        <v>1836.33</v>
+        <v>1836.05</v>
       </c>
       <c r="F1178" s="24" t="n">
-        <v>2186.78</v>
+        <v>2186.45</v>
       </c>
     </row>
     <row r="1179">
@@ -52695,7 +52695,7 @@
     <row r="6">
       <c r="C6" s="28" t="inlineStr">
         <is>
-          <t>Store: Demo Neighbourhood Store (Eden Terrace format).  Data to 25 Sep 2026.  Shelly v1.1.0.</t>
+          <t>Store: Demo Neighbourhood Store (Eden Terrace format).  Data to 25 Sep 2026.  Shelly v1.4.0.</t>
         </is>
       </c>
     </row>
@@ -52818,7 +52818,7 @@
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Generated by Shelly on 29 Sep 2026 22:16</t>
+          <t>Generated by Shelly on 03 Oct 2026 05:37</t>
         </is>
       </c>
     </row>

</xml_diff>